<commit_message>
Add MTL training script, annotated generator output, inference results
</commit_message>
<xml_diff>
--- a/generator/data/kek/kek_adverbs.xlsx
+++ b/generator/data/kek/kek_adverbs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cc6ec0edc09a2fcc/Documents/GitHub/kek-sentence-generator/data/kek/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="373" documentId="8_{D126AFF3-1944-4A81-A981-D2D5BDE9A652}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B30367FC-59BA-4730-9A77-ECE23AB41824}"/>
+  <xr:revisionPtr revIDLastSave="417" documentId="8_{D126AFF3-1944-4A81-A981-D2D5BDE9A652}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78313146-AA4D-4D46-BA2F-54219BFFED49}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{BC957657-B535-49FA-B9D3-4E3FC02517FA}"/>
+    <workbookView xWindow="43080" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{BC957657-B535-49FA-B9D3-4E3FC02517FA}"/>
   </bookViews>
   <sheets>
     <sheet name="semantics_adverbs" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="To add" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">semantics_adverbs!$A$1:$J$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">semantics_adverbs!$A$1:$J$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Verb categories'!$A$1:$E$20</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="276">
   <si>
     <t>lemma_kek</t>
   </si>
@@ -359,9 +359,6 @@
     <t>v_action;v_commerce;v_communicative;v_consumption;v_creation;v_motion;v_ritual;v_sleep</t>
   </si>
   <si>
-    <t>chi x- b’een li ninq’e</t>
-  </si>
-  <si>
     <t>after the fiesta</t>
   </si>
   <si>
@@ -371,15 +368,6 @@
     <t>during the fiesta</t>
   </si>
   <si>
-    <t>chi r-ub’el li ninq’e</t>
-  </si>
-  <si>
-    <t>chi  r-u li ninq’e</t>
-  </si>
-  <si>
-    <t xml:space="preserve">chi r-ix li ninq’e </t>
-  </si>
-  <si>
     <t>r-ix kab’l</t>
   </si>
   <si>
@@ -1953,6 +1941,60 @@
   </si>
   <si>
     <t>sa jun chiab'</t>
+  </si>
+  <si>
+    <t>chi xb’een li ninq’e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chi rix li ninq’e </t>
+  </si>
+  <si>
+    <t>chi rub’el li ninq’e</t>
+  </si>
+  <si>
+    <t>chi  ru li ninq’e</t>
+  </si>
+  <si>
+    <t>mawae'</t>
+  </si>
+  <si>
+    <t>far away</t>
+  </si>
+  <si>
+    <t>distance</t>
+  </si>
+  <si>
+    <t>lejos</t>
+  </si>
+  <si>
+    <t>again</t>
+  </si>
+  <si>
+    <t>otra vez</t>
+  </si>
+  <si>
+    <t>repetition</t>
+  </si>
+  <si>
+    <t>every day</t>
+  </si>
+  <si>
+    <t>cada día</t>
+  </si>
+  <si>
+    <t>hulajhulaj</t>
+  </si>
+  <si>
+    <t>two days ago</t>
+  </si>
+  <si>
+    <t>hace dos días</t>
+  </si>
+  <si>
+    <t>kab'ajer</t>
+  </si>
+  <si>
+    <t>jun sut chik</t>
   </si>
 </sst>
 </file>
@@ -2450,7 +2492,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2470,6 +2512,9 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2526,6 +2571,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2845,7 +2894,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B234044-AE03-447D-83BB-708A3B745400}">
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="19.86328125" customWidth="1"/>
@@ -2881,10 +2930,10 @@
         <v>32</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.45">
@@ -2895,13 +2944,13 @@
         <v>86</v>
       </c>
       <c r="C2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D2" t="s">
         <v>92</v>
       </c>
       <c r="E2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="I2">
         <v>562341.32519034902</v>
@@ -2911,83 +2960,77 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>84</v>
+      <c r="A3" s="1" t="s">
+        <v>259</v>
       </c>
       <c r="B3" t="s">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="C3" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="D3" t="s">
-        <v>92</v>
+        <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="I3">
-        <v>100000</v>
+        <v>1288249.5516931301</v>
       </c>
       <c r="J3">
-        <v>0.29418185562966798</v>
+        <v>3.78979643631174</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>78</v>
+      <c r="A4" s="1" t="s">
+        <v>258</v>
       </c>
       <c r="B4" t="s">
-        <v>87</v>
+        <v>106</v>
       </c>
       <c r="C4" t="s">
         <v>116</v>
       </c>
       <c r="D4" t="s">
-        <v>93</v>
+        <v>9</v>
       </c>
       <c r="E4" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="I4">
-        <v>288403.15031265997</v>
+        <v>1288249.5516931301</v>
       </c>
       <c r="J4">
-        <v>0.84842973928420495</v>
+        <v>3.78979643631174</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>79</v>
+        <v>275</v>
       </c>
       <c r="B5" t="s">
-        <v>88</v>
+        <v>266</v>
       </c>
       <c r="C5" t="s">
-        <v>117</v>
+        <v>267</v>
       </c>
       <c r="D5" t="s">
-        <v>93</v>
+        <v>268</v>
       </c>
       <c r="E5" t="s">
-        <v>102</v>
-      </c>
-      <c r="I5">
-        <v>616595.00186148204</v>
-      </c>
-      <c r="J5">
-        <v>1.8139106181958899</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C6" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="D6" t="s">
         <v>93</v>
@@ -2996,582 +3039,594 @@
         <v>102</v>
       </c>
       <c r="I6">
-        <v>616595.00186148204</v>
+        <v>288403.15031265997</v>
       </c>
       <c r="J6">
-        <v>1.8139106181958899</v>
+        <v>0.84842973928420495</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>81</v>
+      <c r="A7" s="1" t="s">
+        <v>153</v>
       </c>
       <c r="B7" t="s">
-        <v>88</v>
-      </c>
-      <c r="C7" t="s">
-        <v>117</v>
+        <v>154</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>155</v>
       </c>
       <c r="D7" t="s">
-        <v>93</v>
+        <v>9</v>
       </c>
       <c r="E7" t="s">
-        <v>102</v>
+        <v>156</v>
       </c>
       <c r="I7">
-        <v>616595.00186148204</v>
+        <v>407380.27780411299</v>
       </c>
       <c r="J7">
-        <v>1.8139106181958899</v>
+        <v>1.19843886071343</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>83</v>
+      <c r="A8" s="1" t="s">
+        <v>260</v>
       </c>
       <c r="B8" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="C8" t="s">
-        <v>118</v>
+        <v>160</v>
       </c>
       <c r="D8" t="s">
-        <v>93</v>
+        <v>9</v>
       </c>
       <c r="E8" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="I8">
-        <v>288403.15031265997</v>
+        <v>851138.03820237506</v>
       </c>
       <c r="J8">
-        <v>0.84842973928420495</v>
+        <v>2.5038936747537002</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>81</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>57</v>
+        <v>88</v>
+      </c>
+      <c r="C9" t="s">
+        <v>113</v>
       </c>
       <c r="D9" t="s">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="E9" t="s">
-        <v>125</v>
+        <v>102</v>
       </c>
       <c r="I9">
-        <v>933254.30079699005</v>
+        <v>616595.00186148204</v>
       </c>
       <c r="J9">
-        <v>2.7454648198282698</v>
+        <v>1.8139106181958899</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A10" s="1" t="s">
-        <v>141</v>
+      <c r="A10" t="s">
+        <v>79</v>
       </c>
       <c r="B10" t="s">
-        <v>142</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>143</v>
+        <v>88</v>
+      </c>
+      <c r="C10" t="s">
+        <v>113</v>
       </c>
       <c r="D10" t="s">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="E10" t="s">
-        <v>139</v>
+        <v>102</v>
       </c>
       <c r="I10">
-        <v>28840.315031266</v>
+        <v>616595.00186148204</v>
       </c>
       <c r="J10">
-        <v>8.4842973928420495E-2</v>
+        <v>1.8139106181958899</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A11" s="1" t="s">
-        <v>144</v>
+      <c r="A11" t="s">
+        <v>80</v>
       </c>
       <c r="B11" t="s">
-        <v>145</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>146</v>
+        <v>88</v>
+      </c>
+      <c r="C11" t="s">
+        <v>113</v>
       </c>
       <c r="D11" t="s">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="E11" t="s">
-        <v>125</v>
+        <v>102</v>
       </c>
       <c r="I11">
-        <v>501187.23362727201</v>
+        <v>616595.00186148204</v>
       </c>
       <c r="J11">
-        <v>1.47440190406371</v>
+        <v>1.8139106181958899</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A12" s="1" t="s">
-        <v>149</v>
+      <c r="A12" t="s">
+        <v>84</v>
       </c>
       <c r="B12" t="s">
-        <v>150</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>152</v>
+        <v>91</v>
+      </c>
+      <c r="C12" t="s">
+        <v>100</v>
       </c>
       <c r="D12" t="s">
-        <v>11</v>
+        <v>92</v>
       </c>
       <c r="E12" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="I12">
-        <v>478.63009232263801</v>
+        <v>100000</v>
       </c>
       <c r="J12">
-        <v>1.4080428871967299E-3</v>
+        <v>0.29418185562966798</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
-        <v>138</v>
+        <v>261</v>
       </c>
       <c r="B13" t="s">
-        <v>136</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>137</v>
+        <v>108</v>
+      </c>
+      <c r="C13" t="s">
+        <v>117</v>
       </c>
       <c r="D13" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E13" t="s">
-        <v>125</v>
-      </c>
-      <c r="F13" t="s">
-        <v>139</v>
+        <v>102</v>
       </c>
       <c r="I13">
-        <v>245470.891568502</v>
+        <v>630957.34448019299</v>
       </c>
       <c r="J13">
-        <v>0.72213082384691196</v>
+        <v>1.8561620242235</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A14" s="1" t="s">
-        <v>153</v>
+      <c r="A14" t="s">
+        <v>162</v>
       </c>
       <c r="B14" t="s">
-        <v>154</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>155</v>
+        <v>163</v>
+      </c>
+      <c r="C14" t="s">
+        <v>164</v>
       </c>
       <c r="D14" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E14" t="s">
-        <v>156</v>
+        <v>121</v>
+      </c>
+      <c r="G14" t="s">
+        <v>96</v>
       </c>
       <c r="I14">
-        <v>173780.08287493701</v>
+        <v>660693.44800759596</v>
       </c>
       <c r="J14">
-        <v>0.51122947251626605</v>
+        <v>1.94364024537238</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A15" s="1" t="s">
-        <v>130</v>
+      <c r="A15" t="s">
+        <v>271</v>
       </c>
       <c r="B15" t="s">
-        <v>131</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>132</v>
+        <v>269</v>
+      </c>
+      <c r="C15" t="s">
+        <v>270</v>
       </c>
       <c r="D15" t="s">
-        <v>11</v>
+        <v>268</v>
       </c>
       <c r="E15" t="s">
-        <v>125</v>
-      </c>
-      <c r="I15">
-        <v>50118.7233627272</v>
-      </c>
-      <c r="J15">
-        <v>0.14744019040637099</v>
+        <v>121</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A16" s="1" t="s">
-        <v>148</v>
+      <c r="A16" t="s">
+        <v>262</v>
       </c>
       <c r="B16" t="s">
-        <v>135</v>
+        <v>263</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>140</v>
+        <v>265</v>
       </c>
       <c r="D16" t="s">
-        <v>11</v>
+        <v>264</v>
       </c>
       <c r="E16" t="s">
-        <v>125</v>
-      </c>
-      <c r="F16" t="s">
-        <v>139</v>
-      </c>
-      <c r="I16">
-        <v>51286.138399136398</v>
-      </c>
-      <c r="J16">
-        <v>0.150874513623379</v>
+        <v>170</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A17" s="1" t="s">
-        <v>161</v>
+      <c r="A17" t="s">
+        <v>30</v>
       </c>
       <c r="B17" t="s">
-        <v>162</v>
+        <v>10</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>163</v>
+        <v>57</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
       </c>
       <c r="E17" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I17">
-        <v>17782.794100389201</v>
+        <v>933254.30079699005</v>
       </c>
       <c r="J17">
-        <v>5.23137536673281E-2</v>
+        <v>2.7454648198282698</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="B18" t="s">
-        <v>133</v>
+        <v>158</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>134</v>
+        <v>159</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
       </c>
       <c r="E18" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I18">
-        <v>323593.65692962799</v>
+        <v>17782.794100389201</v>
       </c>
       <c r="J18">
-        <v>0.95195382465548195</v>
+        <v>5.23137536673281E-2</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
-        <v>113</v>
+        <v>137</v>
       </c>
       <c r="B19" t="s">
-        <v>114</v>
-      </c>
-      <c r="C19" t="s">
-        <v>165</v>
+        <v>138</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>139</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
       </c>
       <c r="E19" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="I19">
-        <v>588843.65535558795</v>
+        <v>28840.315031266</v>
       </c>
       <c r="J19">
-        <v>1.7322711920826299</v>
+        <v>8.4842973928420495E-2</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A20" t="s">
-        <v>28</v>
+      <c r="A20" s="1" t="s">
+        <v>140</v>
       </c>
       <c r="B20" t="s">
-        <v>7</v>
+        <v>141</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>55</v>
+        <v>142</v>
       </c>
       <c r="D20" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E20" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="I20">
-        <v>77624.7116628691</v>
+        <v>501187.23362727201</v>
       </c>
       <c r="J20">
-        <v>0.22835781719700701</v>
+        <v>1.47440190406371</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A21" t="s">
-        <v>25</v>
+      <c r="A21" s="1" t="s">
+        <v>145</v>
       </c>
       <c r="B21" t="s">
-        <v>3</v>
+        <v>146</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>53</v>
+        <v>148</v>
       </c>
       <c r="D21" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E21" t="s">
-        <v>125</v>
+        <v>152</v>
       </c>
       <c r="I21">
-        <v>1288249.5516931301</v>
+        <v>478.63009232263801</v>
       </c>
       <c r="J21">
-        <v>3.78979643631174</v>
+        <v>1.4080428871967299E-3</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A22" t="s">
-        <v>26</v>
+      <c r="A22" s="1" t="s">
+        <v>134</v>
       </c>
       <c r="B22" t="s">
-        <v>3</v>
+        <v>132</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>53</v>
+        <v>133</v>
       </c>
       <c r="D22" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E22" t="s">
-        <v>125</v>
+        <v>121</v>
+      </c>
+      <c r="F22" t="s">
+        <v>135</v>
       </c>
       <c r="I22">
-        <v>1288249.5516931301</v>
+        <v>245470.891568502</v>
       </c>
       <c r="J22">
-        <v>3.78979643631174</v>
+        <v>0.72213082384691196</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A23" t="s">
-        <v>27</v>
+      <c r="A23" s="1" t="s">
+        <v>149</v>
       </c>
       <c r="B23" t="s">
-        <v>5</v>
+        <v>150</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>54</v>
+        <v>151</v>
       </c>
       <c r="D23" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E23" t="s">
-        <v>101</v>
+        <v>152</v>
       </c>
       <c r="I23">
-        <v>100000</v>
+        <v>173780.08287493701</v>
       </c>
       <c r="J23">
-        <v>0.29418185562966798</v>
+        <v>0.51122947251626605</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A24" t="s">
-        <v>123</v>
+      <c r="A24" s="1" t="s">
+        <v>126</v>
       </c>
       <c r="B24" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>54</v>
+        <v>128</v>
       </c>
       <c r="D24" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E24" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I24">
-        <v>46773.514128719798</v>
+        <v>50118.7233627272</v>
       </c>
       <c r="J24">
-        <v>0.137599191807072</v>
+        <v>0.14744019040637099</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A25" s="1" t="s">
-        <v>106</v>
+        <v>144</v>
       </c>
       <c r="B25" t="s">
-        <v>107</v>
-      </c>
-      <c r="C25" t="s">
-        <v>120</v>
+        <v>131</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>136</v>
       </c>
       <c r="D25" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E25" t="s">
-        <v>125</v>
+        <v>121</v>
+      </c>
+      <c r="F25" t="s">
+        <v>135</v>
       </c>
       <c r="I25">
-        <v>1288249.5516931301</v>
+        <v>51286.138399136398</v>
       </c>
       <c r="J25">
-        <v>3.78979643631174</v>
+        <v>0.150874513623379</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A26" s="1" t="s">
-        <v>112</v>
+        <v>143</v>
       </c>
       <c r="B26" t="s">
-        <v>107</v>
-      </c>
-      <c r="C26" t="s">
-        <v>120</v>
+        <v>129</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>130</v>
       </c>
       <c r="D26" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E26" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I26">
-        <v>1288249.5516931301</v>
+        <v>323593.65692962799</v>
       </c>
       <c r="J26">
-        <v>3.78979643631174</v>
+        <v>0.95195382465548195</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A27" s="1" t="s">
-        <v>157</v>
+      <c r="A27" t="s">
+        <v>12</v>
       </c>
       <c r="B27" t="s">
-        <v>158</v>
+        <v>13</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>159</v>
+        <v>58</v>
       </c>
       <c r="D27" t="s">
         <v>9</v>
       </c>
       <c r="E27" t="s">
-        <v>160</v>
+        <v>104</v>
+      </c>
+      <c r="F27" t="s">
+        <v>103</v>
+      </c>
+      <c r="G27" t="s">
+        <v>94</v>
+      </c>
+      <c r="H27">
+        <v>3</v>
       </c>
       <c r="I27">
-        <v>407380.27780411299</v>
+        <v>602559.58607435797</v>
       </c>
       <c r="J27">
-        <v>1.19843886071343</v>
+        <v>1.7726209715879899</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A28" s="1" t="s">
-        <v>110</v>
+      <c r="A28" t="s">
+        <v>14</v>
       </c>
       <c r="B28" t="s">
-        <v>108</v>
-      </c>
-      <c r="C28" t="s">
-        <v>164</v>
+        <v>253</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>59</v>
       </c>
       <c r="D28" t="s">
         <v>9</v>
       </c>
       <c r="E28" t="s">
-        <v>125</v>
+        <v>104</v>
+      </c>
+      <c r="F28" t="s">
+        <v>103</v>
+      </c>
+      <c r="G28" t="s">
+        <v>94</v>
+      </c>
+      <c r="H28">
+        <v>2</v>
       </c>
       <c r="I28">
-        <v>851138.03820237506</v>
+        <v>1318256.7385563999</v>
       </c>
       <c r="J28">
-        <v>2.5038936747537002</v>
+        <v>3.87807213544838</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A29" s="1" t="s">
-        <v>111</v>
+        <v>41</v>
       </c>
       <c r="B29" t="s">
-        <v>109</v>
-      </c>
-      <c r="C29" t="s">
-        <v>121</v>
+        <v>42</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>69</v>
       </c>
       <c r="D29" t="s">
         <v>9</v>
       </c>
       <c r="E29" t="s">
-        <v>102</v>
+        <v>121</v>
+      </c>
+      <c r="G29" t="s">
+        <v>96</v>
       </c>
       <c r="I29">
-        <v>630957.34448019299</v>
+        <v>724435.96007499006</v>
       </c>
       <c r="J29">
-        <v>1.8561620242235</v>
+        <v>2.1311591501971998</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A30" t="s">
-        <v>166</v>
+      <c r="A30" s="1" t="s">
+        <v>47</v>
       </c>
       <c r="B30" t="s">
-        <v>167</v>
-      </c>
-      <c r="C30" t="s">
-        <v>168</v>
+        <v>48</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>72</v>
       </c>
       <c r="D30" t="s">
         <v>9</v>
       </c>
       <c r="E30" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="G30" t="s">
         <v>96</v>
       </c>
       <c r="I30">
-        <v>660693.44800759596</v>
+        <v>912010.83935590903</v>
       </c>
       <c r="J30">
-        <v>1.94364024537238</v>
+        <v>2.68297041076092</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A31" t="s">
-        <v>12</v>
+      <c r="A31" s="1" t="s">
+        <v>35</v>
       </c>
       <c r="B31" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="D31" t="s">
         <v>9</v>
@@ -3585,77 +3640,83 @@
       <c r="G31" t="s">
         <v>94</v>
       </c>
-      <c r="H31">
-        <v>3</v>
-      </c>
       <c r="I31">
-        <v>602559.58607435797</v>
+        <v>309029.54325135902</v>
       </c>
       <c r="J31">
-        <v>1.7726209715879899</v>
+        <v>0.90910884478073595</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A32" s="1" t="s">
-        <v>41</v>
+      <c r="A32" t="s">
+        <v>15</v>
       </c>
       <c r="B32" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="D32" t="s">
         <v>9</v>
       </c>
       <c r="E32" t="s">
-        <v>125</v>
+        <v>104</v>
+      </c>
+      <c r="F32" t="s">
+        <v>103</v>
       </c>
       <c r="G32" t="s">
-        <v>96</v>
+        <v>94</v>
+      </c>
+      <c r="H32">
+        <v>0</v>
       </c>
       <c r="I32">
-        <v>724435.96007499006</v>
+        <v>549540.87385762401</v>
       </c>
       <c r="J32">
-        <v>2.1311591501971998</v>
+        <v>1.61664954015785</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A33" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B33" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D33" t="s">
         <v>9</v>
       </c>
       <c r="E33" t="s">
-        <v>125</v>
+        <v>104</v>
+      </c>
+      <c r="F33" t="s">
+        <v>103</v>
       </c>
       <c r="G33" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="I33">
-        <v>912010.83935590903</v>
+        <v>501187.23362727201</v>
       </c>
       <c r="J33">
-        <v>2.68297041076092</v>
+        <v>1.47440190406371</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A34" s="1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B34" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D34" t="s">
         <v>9</v>
@@ -3670,21 +3731,21 @@
         <v>94</v>
       </c>
       <c r="I34">
-        <v>309029.54325135902</v>
+        <v>501187.23362727201</v>
       </c>
       <c r="J34">
-        <v>0.90910884478073595</v>
+        <v>1.47440190406371</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A35" t="s">
-        <v>15</v>
+      <c r="A35" s="1" t="s">
+        <v>257</v>
       </c>
       <c r="B35" t="s">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="D35" t="s">
         <v>9</v>
@@ -3698,130 +3759,109 @@
       <c r="G35" t="s">
         <v>94</v>
       </c>
-      <c r="H35">
-        <v>0</v>
-      </c>
       <c r="I35">
-        <v>549540.87385762401</v>
+        <v>912010.83935590903</v>
       </c>
       <c r="J35">
-        <v>1.61664954015785</v>
+        <v>2.68297041076092</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A36" s="1" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="B36" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="D36" t="s">
         <v>9</v>
       </c>
       <c r="E36" t="s">
-        <v>104</v>
-      </c>
-      <c r="F36" t="s">
-        <v>103</v>
+        <v>121</v>
       </c>
       <c r="G36" t="s">
-        <v>94</v>
+        <v>95</v>
+      </c>
+      <c r="H36">
+        <v>0</v>
       </c>
       <c r="I36">
-        <v>501187.23362727201</v>
+        <v>1513561.2484362</v>
       </c>
       <c r="J36">
-        <v>1.47440190406371</v>
+        <v>4.4526225667411996</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A37" s="1" t="s">
-        <v>39</v>
+        <v>109</v>
       </c>
       <c r="B37" t="s">
-        <v>40</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>68</v>
+        <v>110</v>
+      </c>
+      <c r="C37" t="s">
+        <v>161</v>
       </c>
       <c r="D37" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E37" t="s">
-        <v>104</v>
-      </c>
-      <c r="F37" t="s">
-        <v>103</v>
-      </c>
-      <c r="G37" t="s">
-        <v>94</v>
+        <v>121</v>
       </c>
       <c r="I37">
-        <v>501187.23362727201</v>
+        <v>588843.65535558795</v>
       </c>
       <c r="J37">
-        <v>1.47440190406371</v>
+        <v>1.7322711920826299</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A38" s="1" t="s">
-        <v>261</v>
+      <c r="A38" t="s">
+        <v>27</v>
       </c>
       <c r="B38" t="s">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="D38" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E38" t="s">
-        <v>104</v>
-      </c>
-      <c r="F38" t="s">
-        <v>103</v>
-      </c>
-      <c r="G38" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="I38">
-        <v>912010.83935590903</v>
+        <v>100000</v>
       </c>
       <c r="J38">
-        <v>2.68297041076092</v>
+        <v>0.29418185562966798</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A39" s="1" t="s">
-        <v>33</v>
+      <c r="A39" t="s">
+        <v>119</v>
       </c>
       <c r="B39" t="s">
-        <v>34</v>
+        <v>120</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="D39" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E39" t="s">
-        <v>125</v>
-      </c>
-      <c r="G39" t="s">
-        <v>95</v>
-      </c>
-      <c r="H39">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="I39">
-        <v>1513561.2484362</v>
+        <v>46773.514128719798</v>
       </c>
       <c r="J39">
-        <v>4.4526225667411996</v>
+        <v>0.137599191807072</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.45">
@@ -3832,7 +3872,7 @@
         <v>85</v>
       </c>
       <c r="C40" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D40" t="s">
         <v>9</v>
@@ -3858,34 +3898,25 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="B41" t="s">
-        <v>257</v>
+        <v>7</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D41" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E41" t="s">
-        <v>104</v>
-      </c>
-      <c r="F41" t="s">
-        <v>103</v>
-      </c>
-      <c r="G41" t="s">
-        <v>94</v>
-      </c>
-      <c r="H41">
-        <v>2</v>
+        <v>105</v>
       </c>
       <c r="I41">
-        <v>1318256.7385563999</v>
+        <v>77624.7116628691</v>
       </c>
       <c r="J41">
-        <v>3.87807213544838</v>
+        <v>0.22835781719700701</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.45">
@@ -3919,19 +3950,19 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D43" t="s">
         <v>9</v>
       </c>
       <c r="E43" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="G43" t="s">
         <v>94</v>
@@ -3957,7 +3988,7 @@
         <v>9</v>
       </c>
       <c r="E44" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="G44" t="s">
         <v>95</v>
@@ -3999,8 +4030,8 @@
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A46" s="8" t="s">
-        <v>260</v>
+      <c r="A46" t="s">
+        <v>256</v>
       </c>
       <c r="B46" t="s">
         <v>49</v>
@@ -4038,7 +4069,7 @@
         <v>9</v>
       </c>
       <c r="E47" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="G47" t="s">
         <v>96</v>
@@ -4067,7 +4098,7 @@
         <v>9</v>
       </c>
       <c r="E48" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="G48" t="s">
         <v>97</v>
@@ -4084,45 +4115,36 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
+        <v>83</v>
+      </c>
+      <c r="B49" t="s">
+        <v>90</v>
+      </c>
+      <c r="C49" t="s">
+        <v>114</v>
+      </c>
+      <c r="D49" t="s">
+        <v>93</v>
+      </c>
+      <c r="E49" t="s">
+        <v>102</v>
+      </c>
+      <c r="I49">
+        <v>288403.15031265997</v>
+      </c>
+      <c r="J49">
+        <v>0.84842973928420495</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A50" t="s">
         <v>23</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B50" t="s">
         <v>24</v>
       </c>
-      <c r="C49" s="3" t="s">
+      <c r="C50" s="3" t="s">
         <v>64</v>
-      </c>
-      <c r="D49" t="s">
-        <v>9</v>
-      </c>
-      <c r="E49" t="s">
-        <v>104</v>
-      </c>
-      <c r="F49" t="s">
-        <v>103</v>
-      </c>
-      <c r="G49" t="s">
-        <v>94</v>
-      </c>
-      <c r="H49">
-        <v>1</v>
-      </c>
-      <c r="I49">
-        <v>301995.17204020103</v>
-      </c>
-      <c r="J49">
-        <v>0.88841500101987403</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A50" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B50" t="s">
-        <v>52</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>129</v>
       </c>
       <c r="D50" t="s">
         <v>9</v>
@@ -4137,72 +4159,180 @@
         <v>94</v>
       </c>
       <c r="H50">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I50">
-        <v>549540.87385762401</v>
+        <v>301995.17204020103</v>
       </c>
       <c r="J50">
-        <v>1.61664954015785</v>
+        <v>0.88841500101987403</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A51" t="s">
-        <v>82</v>
+      <c r="A51" s="1" t="s">
+        <v>51</v>
       </c>
       <c r="B51" t="s">
-        <v>89</v>
-      </c>
-      <c r="C51" t="s">
-        <v>122</v>
+        <v>52</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>125</v>
       </c>
       <c r="D51" t="s">
         <v>9</v>
       </c>
       <c r="E51" t="s">
-        <v>125</v>
+        <v>104</v>
+      </c>
+      <c r="F51" t="s">
+        <v>103</v>
+      </c>
+      <c r="G51" t="s">
+        <v>94</v>
+      </c>
+      <c r="H51">
+        <v>0</v>
       </c>
       <c r="I51">
+        <v>549540.87385762401</v>
+      </c>
+      <c r="J51">
+        <v>1.61664954015785</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" s="8" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A52" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>272</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="D52" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E52" t="s">
+        <v>104</v>
+      </c>
+      <c r="F52" t="s">
+        <v>103</v>
+      </c>
+      <c r="G52" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="H52" s="8">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A53" t="s">
+        <v>82</v>
+      </c>
+      <c r="B53" t="s">
+        <v>89</v>
+      </c>
+      <c r="C53" t="s">
+        <v>118</v>
+      </c>
+      <c r="D53" t="s">
+        <v>9</v>
+      </c>
+      <c r="E53" t="s">
+        <v>121</v>
+      </c>
+      <c r="I53">
         <v>269153.48039269098</v>
       </c>
-      <c r="J51">
+      <c r="J53">
         <v>0.79180070311105399</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A52" t="s">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A54" t="s">
+        <v>25</v>
+      </c>
+      <c r="B54" t="s">
+        <v>3</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D54" t="s">
+        <v>4</v>
+      </c>
+      <c r="E54" t="s">
+        <v>121</v>
+      </c>
+      <c r="I54">
+        <v>1288249.5516931301</v>
+      </c>
+      <c r="J54">
+        <v>3.78979643631174</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A55" t="s">
+        <v>26</v>
+      </c>
+      <c r="B55" t="s">
+        <v>3</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D55" t="s">
+        <v>4</v>
+      </c>
+      <c r="E55" t="s">
+        <v>121</v>
+      </c>
+      <c r="I55">
+        <v>1288249.5516931301</v>
+      </c>
+      <c r="J55">
+        <v>3.78979643631174</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A56" t="s">
         <v>29</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B56" t="s">
         <v>8</v>
       </c>
-      <c r="C52" s="3" t="s">
+      <c r="C56" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D52" t="s">
+      <c r="D56" t="s">
         <v>9</v>
       </c>
-      <c r="E52" t="s">
-        <v>125</v>
-      </c>
-      <c r="G52" t="s">
+      <c r="E56" t="s">
+        <v>121</v>
+      </c>
+      <c r="G56" t="s">
         <v>96</v>
       </c>
-      <c r="H52">
+      <c r="H56">
         <v>-1</v>
       </c>
-      <c r="I52">
+      <c r="I56">
         <v>123026.877081238</v>
       </c>
-      <c r="J52">
+      <c r="J56">
         <v>0.36192274992081702</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J52" xr:uid="{8B234044-AE03-447D-83BB-708A3B745400}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H52">
-    <sortCondition ref="D2:D52"/>
-    <sortCondition ref="B2:B52"/>
+  <autoFilter ref="A1:J56" xr:uid="{8B234044-AE03-447D-83BB-708A3B745400}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J56">
+      <sortCondition ref="B1:B56"/>
+    </sortState>
+  </autoFilter>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H56">
+    <sortCondition ref="D2:D56"/>
+    <sortCondition ref="B2:B56"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4218,189 +4348,189 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>169</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A2" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>174</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A3" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="E3" s="6" t="s">
         <v>179</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A4" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>184</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A5" s="5" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D5" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>187</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A6" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>192</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A7" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>197</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A8" s="5" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A9" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="E9" s="6" t="s">
         <v>206</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>208</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A10" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>211</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>213</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A11" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>216</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
@@ -4408,16 +4538,16 @@
         <v>103</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
@@ -4425,84 +4555,84 @@
         <v>101</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A14" s="5" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A15" s="5" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A16" s="5" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A17" s="5" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
@@ -4510,50 +4640,50 @@
         <v>102</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A19" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="E19" s="6" t="s">
         <v>247</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>248</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>249</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>250</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A20" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="E20" s="6" t="s">
         <v>252</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>253</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>254</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>255</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>256</v>
       </c>
     </row>
   </sheetData>

</xml_diff>